<commit_message>
Change Name column color to magenta for better terminal contrast
</commit_message>
<xml_diff>
--- a/gca_tracker_template.xlsx
+++ b/gca_tracker_template.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,25 +424,35 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>First Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Last Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Team Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Start Date</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>End Date</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Reason</t>
         </is>
@@ -456,25 +466,35 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>John</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Doe</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>Engineering</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Provisioned</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Gemini Code Assist access for Q2 Project</t>
         </is>
@@ -488,25 +508,35 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>Jane</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Smith</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>Data Science</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Onboarding new hire</t>
         </is>
@@ -520,25 +550,35 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>Bob</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Johnson</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Provisioned</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Contract ending</t>
         </is>
@@ -552,25 +592,35 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>Alice</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Williams</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>Security</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>2026-08-01</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Future project needs</t>
         </is>

</xml_diff>